<commit_message>
security(S1-07): scrub real name/email from public import template
The bulk-employee-import template's sample row had a real developer name
and @spaculus.com email address, publicly downloadable with no login.
Replaced with obvious placeholder data; column headers and every other
sample value are unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/resorts_assets/demofiles/Employee.xlsx
+++ b/public/resorts_assets/demofiles/Employee.xlsx
@@ -138,7 +138,7 @@
     <t>rooms-director</t>
   </si>
   <si>
-    <t xml:space="preserve">Ashvin </t>
+    <t xml:space="preserve">Jane </t>
   </si>
   <si>
     <t>xxxx</t>
@@ -147,7 +147,7 @@
     <t>xxx</t>
   </si>
   <si>
-    <t>web.ashvin@spaculus.com</t>
+    <t>jane.doe@example.com</t>
   </si>
   <si>
     <t>male</t>

</xml_diff>